<commit_message>
Fix: Vercel build blocker (dynamic routes for latest, sitemap, neighborhoods) + CTA fallback injection
</commit_message>
<xml_diff>
--- a/digital-products/car-vs-mrt-grab-calculator/singapore-car-vs-mrt-grab-decision-calculator-2026.xlsx
+++ b/digital-products/car-vs-mrt-grab-calculator/singapore-car-vs-mrt-grab-decision-calculator-2026.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="87" uniqueCount="87">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="92">
   <si>
     <t>SINGAPORE CAR  vs  MRT + GRAB</t>
   </si>
@@ -202,10 +202,14 @@
     <t>Scenario B · MRT / bus + Grab / taxi</t>
   </si>
   <si>
-    <t>Scenario C · Car ownership</t>
-  </si>
-  <si>
-    <t>Scenario C = loan payment + petrol + parking + ERP + insurance + maintenance + other costs + depreciation (annual ÷ 12). It excludes the upfront cash outlay shown on the INPUTS tab — read both together before deciding.</t>
+    <t>Scenario C · Car ownership — Monthly Cash Outflow</t>
+  </si>
+  <si>
+    <t>Scenario C · Car ownership — Monthly Economic Cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Monthly Cash Outflow = loan payment + petrol + parking + ERP + insurance + maintenance + other costs (excludes depreciation).
+Monthly Economic Cost = Cash Outflow + depreciation (annual ÷ 12). Upfront cash outlay is shown on the INPUTS tab — read both together before deciding.</t>
   </si>
   <si>
     <t>DIFFERENCE BETWEEN SCENARIOS</t>
@@ -214,19 +218,22 @@
     <t>Adding Grab / taxi (B − A)</t>
   </si>
   <si>
-    <t>Owning a car instead of MRT + Grab (C − B)</t>
-  </si>
-  <si>
-    <t>Relative cost — car ÷ MRT + Grab</t>
+    <t>Owning a car instead of MRT + Grab (Economic Cost − B)</t>
+  </si>
+  <si>
+    <t>Car Cash Outflow vs MRT + Grab (Cash Outflow − B)</t>
+  </si>
+  <si>
+    <t>Relative cost — car Economic Cost ÷ MRT + Grab</t>
   </si>
   <si>
     <t>WHICH SCENARIO IS CHEAPER FOR YOU?</t>
   </si>
   <si>
-    <t>Overall verdict</t>
-  </si>
-  <si>
-    <t>Tip: a lower monthly figure is not the whole story — weigh convenience, family needs, reliability and the upfront cash required before committing.</t>
+    <t>Overall verdict (Economic Cost)</t>
+  </si>
+  <si>
+    <t>Tip: Compare Economic Cost (includes depreciation) for true cost of ownership. Cash Outflow shows actual monthly cash spending. Upfront cash required is on the INPUTS tab.</t>
   </si>
   <si>
     <t>STEP 3 · STRESS-TEST YOUR ASSUMPTIONS</t>
@@ -253,13 +260,22 @@
     <t>What this means for you</t>
   </si>
   <si>
-    <t>SENSITIVITY — TOTAL MONTHLY CAR COST UNDER DIFFERENT ASSUMPTIONS</t>
+    <t>SENSITIVITY — MONTHLY ECONOMIC COST (INCLUDES DEPRECIATION)</t>
   </si>
   <si>
     <t>Annual depreciation ↓   /   Petrol →</t>
   </si>
   <si>
-    <t>Each cell is the TOTAL monthly cost of owning a car for that combination of annual depreciation and petrol spend (all other inputs stay as entered on the INPUTS tab). Compare each figure with your monthly MRT + Grab total on the COMPARISON tab — any cell below that figure suggests car ownership could be cheaper under that combination.</t>
+    <t>Each cell is the Monthly Economic Cost (Cash Outflow + depreciation) of owning a car for that combination of annual depreciation and petrol spend (all other inputs stay as entered on the INPUTS tab). Compare with your monthly MRT + Grab total on the COMPARISON tab.</t>
+  </si>
+  <si>
+    <t>SENSITIVITY — MONTHLY CASH OUTFLOW (EXCLUDES DEPRECIATION)</t>
+  </si>
+  <si>
+    <t>Annual depreciation (not in cash outflow) ↓   /   Petrol →</t>
+  </si>
+  <si>
+    <t>Each cell is the Monthly Cash Outflow (excludes depreciation) of owning a car. This represents actual monthly cash spending. Compare with your monthly MRT + Grab total on the COMPARISON tab to understand cash flow impact.</t>
   </si>
   <si>
     <t>TRY THESE QUICK EXPERIMENTS</t>
@@ -1389,7 +1405,7 @@
   <sheetPr>
     <tabColor rgb="FF16A34A"/>
   </sheetPr>
-  <dimension ref="B1:F19"/>
+  <dimension ref="B1:F20"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -1464,71 +1480,71 @@
       </c>
     </row>
     <row r="7" ht="24" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B7" s="17" t="s">
+      <c r="B7" s="16" t="s">
         <v>62</v>
       </c>
-      <c r="C7" s="18">
+      <c r="C7" s="13">
+        <f>INPUTS!C12+INPUTS!C14+INPUTS!C15+INPUTS!C16+INPUTS!C17+INPUTS!C18+INPUTS!C19</f>
+        <v>NaN</v>
+      </c>
+      <c r="D7" s="13">
+        <f>(INPUTS!C12+INPUTS!C14+INPUTS!C15+INPUTS!C16+INPUTS!C17+INPUTS!C18+INPUTS!C19)*12</f>
+        <v>NaN</v>
+      </c>
+      <c r="E7" s="13">
+        <f>(INPUTS!C12+INPUTS!C14+INPUTS!C15+INPUTS!C16+INPUTS!C17+INPUTS!C18+INPUTS!C19)*120</f>
+        <v>NaN</v>
+      </c>
+    </row>
+    <row r="8" ht="24" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B8" s="17" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" s="18">
         <f>INPUTS!C12+INPUTS!C14+INPUTS!C15+INPUTS!C16+INPUTS!C17+INPUTS!C18+INPUTS!C19+INPUTS!C21/12</f>
         <v>3310</v>
       </c>
-      <c r="D7" s="18">
+      <c r="D8" s="18">
         <f>(INPUTS!C12+INPUTS!C14+INPUTS!C15+INPUTS!C16+INPUTS!C17+INPUTS!C18+INPUTS!C19+INPUTS!C21/12)*12</f>
         <v>39720</v>
       </c>
-      <c r="E7" s="18">
+      <c r="E8" s="18">
         <f>(INPUTS!C12+INPUTS!C14+INPUTS!C15+INPUTS!C16+INPUTS!C17+INPUTS!C18+INPUTS!C19+INPUTS!C21/12)*120</f>
         <v>397200</v>
       </c>
     </row>
-    <row r="8" ht="30" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B8" s="19" t="s">
-        <v>63</v>
-      </c>
-      <c r="C8" s="19"/>
-      <c r="D8" s="19"/>
-      <c r="E8" s="19"/>
-    </row>
-    <row r="10" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B10" s="4" t="s">
+    <row r="9" ht="36" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B9" s="19" t="s">
         <v>64</v>
       </c>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="4"/>
-    </row>
-    <row r="11" ht="22" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B11" s="16" t="s">
+      <c r="C9" s="19"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19"/>
+    </row>
+    <row r="11" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B11" s="4" t="s">
         <v>65</v>
       </c>
-      <c r="C11" s="13">
-        <f>INPUTS!C7</f>
-        <v>300</v>
-      </c>
-      <c r="D11" s="13">
-        <f>INPUTS!C7*12</f>
-        <v>3600</v>
-      </c>
-      <c r="E11" s="13">
-        <f>INPUTS!C7*120</f>
-        <v>36000</v>
-      </c>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
+      <c r="F11" s="4"/>
     </row>
     <row r="12" ht="22" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B12" s="16" t="s">
         <v>66</v>
       </c>
       <c r="C12" s="13">
-        <f>C7-C6</f>
-        <v>2890</v>
+        <f>INPUTS!C7</f>
+        <v>300</v>
       </c>
       <c r="D12" s="13">
-        <f>D7-D6</f>
-        <v>34680</v>
+        <f>INPUTS!C7*12</f>
+        <v>3600</v>
       </c>
       <c r="E12" s="13">
-        <f>E7-E6</f>
-        <v>346800</v>
+        <f>INPUTS!C7*120</f>
+        <v>36000</v>
       </c>
     </row>
     <row r="13" ht="22" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
@@ -1536,65 +1552,99 @@
         <v>67</v>
       </c>
       <c r="C13" s="13">
-        <f>IF(C6&gt;0,C7/C6,"n/a")</f>
+        <f>C8-C6</f>
+        <v>2890</v>
+      </c>
+      <c r="D13" s="13">
+        <f>D8-D6</f>
+        <v>34680</v>
+      </c>
+      <c r="E13" s="13">
+        <f>E8-E6</f>
+        <v>346800</v>
+      </c>
+    </row>
+    <row r="14" ht="22" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B14" s="16" t="s">
+        <v>68</v>
+      </c>
+      <c r="C14" s="13">
+        <f>C7-C6</f>
+        <v>NaN</v>
+      </c>
+      <c r="D14" s="13">
+        <f>D7-D6</f>
+        <v>NaN</v>
+      </c>
+      <c r="E14" s="13">
+        <f>E7-E6</f>
+        <v>NaN</v>
+      </c>
+    </row>
+    <row r="15" ht="22" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B15" s="16" t="s">
+        <v>69</v>
+      </c>
+      <c r="C15" s="13">
+        <f>IF(C6&gt;0,C8/C6,"n/a")</f>
         <v>7.880952380952381</v>
       </c>
-      <c r="D13" s="13">
-        <f>IF(D6&gt;0,D7/D6,"n/a")</f>
+      <c r="D15" s="13">
+        <f>IF(D6&gt;0,D8/D6,"n/a")</f>
         <v>7.880952380952381</v>
       </c>
-      <c r="E13" s="13">
-        <f>IF(E6&gt;0,E7/E6,"n/a")</f>
+      <c r="E15" s="13">
+        <f>IF(E6&gt;0,E8/E6,"n/a")</f>
         <v>7.880952380952381</v>
       </c>
     </row>
-    <row r="15" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
-      <c r="B15" s="4" t="s">
-        <v>68</v>
-      </c>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-    </row>
-    <row r="16" ht="26" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B16" s="20" t="s">
-        <v>69</v>
-      </c>
-      <c r="C16" s="21" t="str">
-        <f>IF(C7&gt;C6,"Under your current assumptions, MRT + Grab is CHEAPER than owning a car.","Under your current assumptions, owning a car is CHEAPER than MRT + Grab.")</f>
-        <v>Under your current assumptions, MRT + Grab is CHEAPER than owning a car.</v>
-      </c>
-      <c r="D16" s="21"/>
-      <c r="E16" s="21"/>
-    </row>
-    <row r="17" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B17" s="22" t="str">
-        <f>"At your assumed Grab / taxi spend, a car costs about "&amp;TEXT(MAX(0,C7-C6),"S$#,##0")&amp;" more (or less) per month than MRT + Grab."</f>
-        <v>At your assumed Grab / taxi spend, a car costs about S$2,890 more (or less) per month than MRT + Grab.</v>
-      </c>
-      <c r="C17" s="22"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="22"/>
-    </row>
-    <row r="19" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B19" s="23" t="s">
+    <row r="16" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B16" s="4" t="s">
         <v>70</v>
       </c>
-      <c r="C19" s="23"/>
-      <c r="D19" s="23"/>
-      <c r="E19" s="23"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4"/>
+    </row>
+    <row r="17" ht="26" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B17" s="20" t="s">
+        <v>71</v>
+      </c>
+      <c r="C17" s="21" t="str">
+        <f>IF(C8&gt;C6,"Under your current assumptions, MRT + Grab is CHEAPER than owning a car (Economic Cost).","Under your current assumptions, owning a car is CHEAPER than MRT + Grab (Economic Cost).")</f>
+        <v>Under your current assumptions, MRT + Grab is CHEAPER than owning a car (Economic Cost).</v>
+      </c>
+      <c r="D17" s="21"/>
+      <c r="E17" s="21"/>
+    </row>
+    <row r="18" ht="22" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B18" s="22" t="str">
+        <f>"At your assumed Grab / taxi spend, a car (Economic Cost) costs about "&amp;TEXT(MAX(0,C8-C6),"S$#,##0")&amp;" more (or less) per month than MRT + Grab. Cash Outflow difference: "&amp;TEXT(MAX(0,C7-C6),"S$#,##0")</f>
+        <v>At your assumed Grab / taxi spend, a car (Economic Cost) costs about S$2,890 more (or less) per month than MRT + Grab. Cash Outflow difference: S$NaN</v>
+      </c>
+      <c r="C18" s="22"/>
+      <c r="D18" s="22"/>
+      <c r="E18" s="22"/>
+    </row>
+    <row r="20" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B20" s="23" t="s">
+        <v>72</v>
+      </c>
+      <c r="C20" s="23"/>
+      <c r="D20" s="23"/>
+      <c r="E20" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="8">
     <mergeCell ref="B1:F1"/>
     <mergeCell ref="B2:F2"/>
-    <mergeCell ref="B8:E8"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="B15:F15"/>
-    <mergeCell ref="C16:E16"/>
-    <mergeCell ref="B17:E17"/>
-    <mergeCell ref="B19:E19"/>
+    <mergeCell ref="B9:E9"/>
+    <mergeCell ref="B11:F11"/>
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="C17:E17"/>
+    <mergeCell ref="B18:E18"/>
+    <mergeCell ref="B20:E20"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
@@ -1606,7 +1656,7 @@
   <sheetPr>
     <tabColor rgb="FF9333EA"/>
   </sheetPr>
-  <dimension ref="B1:F22"/>
+  <dimension ref="B1:F31"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="3" customWidth="1"/>
@@ -1616,7 +1666,7 @@
   <sheetData>
     <row r="1" ht="34" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B1" s="8" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C1" s="8"/>
       <c r="D1" s="8"/>
@@ -1625,7 +1675,7 @@
     </row>
     <row r="2" ht="20" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B2" s="9" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="C2" s="9"/>
       <c r="D2" s="9"/>
@@ -1634,7 +1684,7 @@
     </row>
     <row r="4" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B4" s="4" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C4" s="4"/>
       <c r="D4" s="4"/>
@@ -1643,35 +1693,35 @@
     </row>
     <row r="5" ht="22" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B5" s="10" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="C5" s="13">
         <f>INPUTS!C7</f>
         <v>300</v>
       </c>
       <c r="D5" s="12" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="E5" s="12"/>
       <c r="F5" s="12"/>
     </row>
     <row r="6" ht="22" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B6" s="10" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="C6" s="18">
         <f>MAX(0,(INPUTS!C12+INPUTS!C14+INPUTS!C15+INPUTS!C16+INPUTS!C17+INPUTS!C18+INPUTS!C19+INPUTS!C21/12)-INPUTS!C5)</f>
         <v>3190</v>
       </c>
       <c r="D6" s="12" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="E6" s="12"/>
       <c r="F6" s="12"/>
     </row>
     <row r="7" ht="22" customHeight="1" spans="2:3" x14ac:dyDescent="0.25">
       <c r="B7" s="10" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="C7" s="24" t="str">
         <f>IF(INPUTS!C7&gt;=MAX(0,(INPUTS!C12+INPUTS!C14+INPUTS!C15+INPUTS!C16+INPUTS!C17+INPUTS!C18+INPUTS!C19+INPUTS!C21/12)-INPUTS!C5),"Your Grab / taxi spending is AT or ABOVE break-even — under your assumptions, a car may be financially rational.","A car only becomes cost-comparable if your monthly Grab / taxi spend rises to the break-even level above.")</f>
@@ -1680,7 +1730,7 @@
     </row>
     <row r="9" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B9" s="4" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C9" s="4"/>
       <c r="D9" s="4"/>
@@ -1689,7 +1739,7 @@
     </row>
     <row r="10" ht="26" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B10" s="25" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="C10" s="26">
         <v>150</v>
@@ -1788,7 +1838,7 @@
     </row>
     <row r="16" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
       <c r="B16" s="19" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="C16" s="19"/>
       <c r="D16" s="19"/>
@@ -1796,47 +1846,163 @@
     </row>
     <row r="18" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
       <c r="B18" s="4" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="C18" s="4"/>
       <c r="D18" s="4"/>
       <c r="E18" s="4"/>
       <c r="F18" s="4"/>
     </row>
-    <row r="19" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B19" s="28" t="s">
-        <v>83</v>
-      </c>
-      <c r="C19" s="28"/>
-      <c r="D19" s="28"/>
-      <c r="E19" s="28"/>
-    </row>
-    <row r="20" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B20" s="28" t="s">
-        <v>84</v>
-      </c>
-      <c r="C20" s="28"/>
-      <c r="D20" s="28"/>
-      <c r="E20" s="28"/>
-    </row>
-    <row r="21" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B21" s="28" t="s">
+    <row r="19" ht="26" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B19" s="25" t="s">
         <v>85</v>
       </c>
-      <c r="C21" s="28"/>
-      <c r="D21" s="28"/>
-      <c r="E21" s="28"/>
-    </row>
-    <row r="22" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
-      <c r="B22" s="28" t="s">
+      <c r="C19" s="26">
+        <v>150</v>
+      </c>
+      <c r="D19" s="26">
+        <v>250</v>
+      </c>
+      <c r="E19" s="26">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="20" ht="22" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B20" s="27">
+        <v>6000</v>
+      </c>
+      <c r="C20" s="13">
+        <f>INPUTS!C12+INPUTS!C15+INPUTS!C16+INPUTS!C17+INPUTS!C18+INPUTS!C19+C$19</f>
+        <v>2210</v>
+      </c>
+      <c r="D20" s="13">
+        <f>INPUTS!C12+INPUTS!C15+INPUTS!C16+INPUTS!C17+INPUTS!C18+INPUTS!C19+D$19</f>
+        <v>2310</v>
+      </c>
+      <c r="E20" s="13">
+        <f>INPUTS!C12+INPUTS!C15+INPUTS!C16+INPUTS!C17+INPUTS!C18+INPUTS!C19+E$19</f>
+        <v>2410</v>
+      </c>
+    </row>
+    <row r="21" ht="22" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B21" s="27">
+        <v>9000</v>
+      </c>
+      <c r="C21" s="13">
+        <f>INPUTS!C12+INPUTS!C15+INPUTS!C16+INPUTS!C17+INPUTS!C18+INPUTS!C19+C$19</f>
+        <v>2210</v>
+      </c>
+      <c r="D21" s="13">
+        <f>INPUTS!C12+INPUTS!C15+INPUTS!C16+INPUTS!C17+INPUTS!C18+INPUTS!C19+D$19</f>
+        <v>2310</v>
+      </c>
+      <c r="E21" s="13">
+        <f>INPUTS!C12+INPUTS!C15+INPUTS!C16+INPUTS!C17+INPUTS!C18+INPUTS!C19+E$19</f>
+        <v>2410</v>
+      </c>
+    </row>
+    <row r="22" ht="22" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B22" s="27">
+        <v>12000</v>
+      </c>
+      <c r="C22" s="13">
+        <f>INPUTS!C12+INPUTS!C15+INPUTS!C16+INPUTS!C17+INPUTS!C18+INPUTS!C19+C$19</f>
+        <v>2210</v>
+      </c>
+      <c r="D22" s="13">
+        <f>INPUTS!C12+INPUTS!C15+INPUTS!C16+INPUTS!C17+INPUTS!C18+INPUTS!C19+D$19</f>
+        <v>2310</v>
+      </c>
+      <c r="E22" s="13">
+        <f>INPUTS!C12+INPUTS!C15+INPUTS!C16+INPUTS!C17+INPUTS!C18+INPUTS!C19+E$19</f>
+        <v>2410</v>
+      </c>
+    </row>
+    <row r="23" ht="22" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B23" s="27">
+        <v>15000</v>
+      </c>
+      <c r="C23" s="13">
+        <f>INPUTS!C12+INPUTS!C15+INPUTS!C16+INPUTS!C17+INPUTS!C18+INPUTS!C19+C$19</f>
+        <v>2210</v>
+      </c>
+      <c r="D23" s="13">
+        <f>INPUTS!C12+INPUTS!C15+INPUTS!C16+INPUTS!C17+INPUTS!C18+INPUTS!C19+D$19</f>
+        <v>2310</v>
+      </c>
+      <c r="E23" s="13">
+        <f>INPUTS!C12+INPUTS!C15+INPUTS!C16+INPUTS!C17+INPUTS!C18+INPUTS!C19+E$19</f>
+        <v>2410</v>
+      </c>
+    </row>
+    <row r="24" ht="22" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B24" s="27">
+        <v>18000</v>
+      </c>
+      <c r="C24" s="13">
+        <f>INPUTS!C12+INPUTS!C15+INPUTS!C16+INPUTS!C17+INPUTS!C18+INPUTS!C19+C$19</f>
+        <v>2210</v>
+      </c>
+      <c r="D24" s="13">
+        <f>INPUTS!C12+INPUTS!C15+INPUTS!C16+INPUTS!C17+INPUTS!C18+INPUTS!C19+D$19</f>
+        <v>2310</v>
+      </c>
+      <c r="E24" s="13">
+        <f>INPUTS!C12+INPUTS!C15+INPUTS!C16+INPUTS!C17+INPUTS!C18+INPUTS!C19+E$19</f>
+        <v>2410</v>
+      </c>
+    </row>
+    <row r="25" ht="44" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B25" s="19" t="s">
         <v>86</v>
       </c>
-      <c r="C22" s="28"/>
-      <c r="D22" s="28"/>
-      <c r="E22" s="28"/>
+      <c r="C25" s="19"/>
+      <c r="D25" s="19"/>
+      <c r="E25" s="19"/>
+    </row>
+    <row r="27" ht="24" customHeight="1" spans="2:6" x14ac:dyDescent="0.25">
+      <c r="B27" s="4" t="s">
+        <v>87</v>
+      </c>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4"/>
+    </row>
+    <row r="28" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B28" s="28" t="s">
+        <v>88</v>
+      </c>
+      <c r="C28" s="28"/>
+      <c r="D28" s="28"/>
+      <c r="E28" s="28"/>
+    </row>
+    <row r="29" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B29" s="28" t="s">
+        <v>89</v>
+      </c>
+      <c r="C29" s="28"/>
+      <c r="D29" s="28"/>
+      <c r="E29" s="28"/>
+    </row>
+    <row r="30" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B30" s="28" t="s">
+        <v>90</v>
+      </c>
+      <c r="C30" s="28"/>
+      <c r="D30" s="28"/>
+      <c r="E30" s="28"/>
+    </row>
+    <row r="31" ht="20" customHeight="1" spans="2:5" x14ac:dyDescent="0.25">
+      <c r="B31" s="28" t="s">
+        <v>91</v>
+      </c>
+      <c r="C31" s="28"/>
+      <c r="D31" s="28"/>
+      <c r="E31" s="28"/>
     </row>
   </sheetData>
-  <mergeCells count="12">
+  <mergeCells count="14">
     <mergeCell ref="B1:F1"/>
     <mergeCell ref="B2:F2"/>
     <mergeCell ref="B4:F4"/>
@@ -1845,10 +2011,12 @@
     <mergeCell ref="B9:F9"/>
     <mergeCell ref="B16:E16"/>
     <mergeCell ref="B18:F18"/>
-    <mergeCell ref="B19:E19"/>
-    <mergeCell ref="B20:E20"/>
-    <mergeCell ref="B21:E21"/>
-    <mergeCell ref="B22:E22"/>
+    <mergeCell ref="B25:E25"/>
+    <mergeCell ref="B27:F27"/>
+    <mergeCell ref="B28:E28"/>
+    <mergeCell ref="B29:E29"/>
+    <mergeCell ref="B30:E30"/>
+    <mergeCell ref="B31:E31"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>